<commit_message>
Fixed bugs, finished plots, fix def
</commit_message>
<xml_diff>
--- a/data/parrotfish data/parrotfish_metadata.xlsx
+++ b/data/parrotfish data/parrotfish_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JonathanB22\Desktop\Dan\Eilat_2017_MHW\Red_Sea_MHWs_Parrotfish\data\parrotfish data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{219A8B13-2D57-4C26-AE78-4A3740413C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E95CA0-4DEA-400E-AB0C-0A3AB45B34B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{FB66EAEE-B1FF-4CD3-9195-8C463EB6069F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{FB66EAEE-B1FF-4CD3-9195-8C463EB6069F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>